<commit_message>
fix: preserve cached formula values on save without EvaluateFormulasBeforeSaving
Previously, WriteCellWithFormula only wrote cached values to the XML when
EvaluateFormulasBeforeSaving was true. This caused formula cells loaded
from Excel files to lose their cached results on round-trip, particularly
affecting:

- Dynamic array formulas (SORT, UNIQUE, FILTER) that XLibur cannot evaluate
- Spill (non-master) cells of array formulas losing both values and type attributes
- Any formula cell with a pre-computed cached value

Now cached values are always written when they exist and the formula has not
been dirtied (NeedsRecalculation is false). The EvaluateFormulasBeforeSaving
flag now only controls whether formulas are re-evaluated during save, not
whether existing cached results are preserved.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/Misc/CopyingWorksheets.xlsx
+++ b/XLibur.Tests/Resource/Examples/Misc/CopyingWorksheets.xlsx
@@ -946,7 +946,7 @@
       </x:c>
     </x:row>
     <x:row r="9" spans="1:11">
-      <x:c r="I9" s="0">
+      <x:c r="I9" s="0" t="str">
         <x:f>CONCATENATE("Count: ", CountA(Headers[Table Headers]))</x:f>
       </x:c>
     </x:row>
@@ -1114,7 +1114,7 @@
       </x:c>
     </x:row>
     <x:row r="9" spans="1:11">
-      <x:c r="I9" s="0">
+      <x:c r="I9" s="0" t="str">
         <x:f>CONCATENATE("Count: ", CountA(Headers[Table Headers]))</x:f>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
fix: preserve cached formula values on save without EvaluateFormulasBeforeSaving (#54)
Previously, WriteCellWithFormula only wrote cached values to the XML when
EvaluateFormulasBeforeSaving was true. This caused formula cells loaded
from Excel files to lose their cached results on round-trip, particularly
affecting:

- Dynamic array formulas (SORT, UNIQUE, FILTER) that XLibur cannot evaluate
- Spill (non-master) cells of array formulas losing both values and type attributes
- Any formula cell with a pre-computed cached value

Now cached values are always written when they exist and the formula has not
been dirtied (NeedsRecalculation is false). The EvaluateFormulasBeforeSaving
flag now only controls whether formulas are re-evaluated during save, not
whether existing cached results are preserved.
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/Misc/CopyingWorksheets.xlsx
+++ b/XLibur.Tests/Resource/Examples/Misc/CopyingWorksheets.xlsx
@@ -946,7 +946,7 @@
       </x:c>
     </x:row>
     <x:row r="9" spans="1:11">
-      <x:c r="I9" s="0">
+      <x:c r="I9" s="0" t="str">
         <x:f>CONCATENATE("Count: ", CountA(Headers[Table Headers]))</x:f>
       </x:c>
     </x:row>
@@ -1114,7 +1114,7 @@
       </x:c>
     </x:row>
     <x:row r="9" spans="1:11">
-      <x:c r="I9" s="0">
+      <x:c r="I9" s="0" t="str">
         <x:f>CONCATENATE("Count: ", CountA(Headers[Table Headers]))</x:f>
       </x:c>
     </x:row>

</xml_diff>